<commit_message>
Restrict ⑯ to 18 countries; discount messages-per-user by AEI 18-country share; update reports 17-18
- 02_clean_sensortower_share_all_products.do: part 2 (⑯) now sums the 18
  country sheets instead of the 25-market Worldwide row.
- 03_merge_sensortower_openai_messages.do: msgs_per_user = ChatGPT global
  monthly messages × 18-country share (AEI Claude.ai 2025-08-04..11, 61.01%)
  ÷ 18-country ChatGPT users → 53.75 (was 80.20). Adds assumption (A3).
- 04_analysis_sensortower_messages_summary.do: anchor table shows the
  discount steps; rerun tables. Report 18 tables unchanged (normalized shares).
- Reports 17 and 18 (.tex/.md) updated; log.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/table/17_sensortower_messages.xlsx
+++ b/results/table/17_sensortower_messages.xlsx
@@ -15,7 +15,874 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="417">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>2024-07</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>assistant</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>DeepSeek</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Grok</t>
+  </si>
+  <si>
+    <t>Microsoft Copilot</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Perplexity</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>DeepSeek</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Grok</t>
+  </si>
+  <si>
+    <t>Microsoft Copilot</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Perplexity</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>DeepSeek</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Grok</t>
+  </si>
+  <si>
+    <t>Microsoft Copilot</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Perplexity</t>
+  </si>
+  <si>
+    <t>unique_users</t>
+  </si>
+  <si>
+    <t>share_ww_pct</t>
+  </si>
+  <si>
+    <t>msgs_per_user</t>
+  </si>
+  <si>
+    <t>messages</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>market</t>
+  </si>
+  <si>
+    <t>Argentina</t>
+  </si>
+  <si>
+    <t>Australia</t>
+  </si>
+  <si>
+    <t>Brazil</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Indonesia</t>
+  </si>
+  <si>
+    <t>Italy</t>
+  </si>
+  <si>
+    <t>Japan</t>
+  </si>
+  <si>
+    <t>Mexico</t>
+  </si>
+  <si>
+    <t>South Korea</t>
+  </si>
+  <si>
+    <t>Spain</t>
+  </si>
+  <si>
+    <t>Taiwan</t>
+  </si>
+  <si>
+    <t>Turkey</t>
+  </si>
+  <si>
+    <t>United Kingdom</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>Vietnam</t>
+  </si>
+  <si>
+    <t>Other 7 markets (residual)</t>
+  </si>
+  <si>
+    <t>iso2</t>
+  </si>
+  <si>
+    <t>AR</t>
+  </si>
+  <si>
+    <t>AU</t>
+  </si>
+  <si>
+    <t>BR</t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t>FR</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>JP</t>
+  </si>
+  <si>
+    <t>MX</t>
+  </si>
+  <si>
+    <t>KR</t>
+  </si>
+  <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>TW</t>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+  <si>
+    <t>GB</t>
+  </si>
+  <si>
+    <t>US</t>
+  </si>
+  <si>
+    <t>VN</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>residual</t>
+  </si>
+  <si>
+    <t>all_users</t>
+  </si>
+  <si>
+    <t>messages</t>
+  </si>
+  <si>
+    <t>work_share</t>
+  </si>
+  <si>
+    <t>work_share_src</t>
+  </si>
+  <si>
+    <t>Signals 국가별</t>
+  </si>
+  <si>
+    <t>Signals 전 세계(residual)</t>
+  </si>
+  <si>
+    <t>work_messages</t>
+  </si>
+  <si>
+    <t>nonwork_messages</t>
+  </si>
+  <si>
+    <t>conv_k1p5</t>
+  </si>
+  <si>
+    <t>conv_k3</t>
+  </si>
+  <si>
+    <t>conv_k5</t>
+  </si>
+  <si>
+    <t>conv_k7</t>
+  </si>
+  <si>
+    <t>conv_k10</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>2024-07</t>
+  </si>
+  <si>
+    <t>2024-08</t>
+  </si>
+  <si>
+    <t>2024-09</t>
+  </si>
+  <si>
+    <t>2024-10</t>
+  </si>
+  <si>
+    <t>2024-11</t>
+  </si>
+  <si>
+    <t>2024-12</t>
+  </si>
+  <si>
+    <t>2025-01</t>
+  </si>
+  <si>
+    <t>2025-02</t>
+  </si>
+  <si>
+    <t>2025-03</t>
+  </si>
+  <si>
+    <t>2025-04</t>
+  </si>
+  <si>
+    <t>2025-05</t>
+  </si>
+  <si>
+    <t>2025-06</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>market</t>
+  </si>
+  <si>
+    <t>Worldwide</t>
+  </si>
+  <si>
+    <t>worldwide_users</t>
+  </si>
+  <si>
+    <t>msgs_per_user</t>
+  </si>
+  <si>
+    <t>messages</t>
+  </si>
+  <si>
+    <t>work_share_implied</t>
+  </si>
+  <si>
+    <t>work_messages</t>
+  </si>
+  <si>
+    <t>nonwork_messages</t>
+  </si>
+  <si>
+    <t>work_share_global</t>
+  </si>
+  <si>
+    <t>work_messages_global</t>
+  </si>
+  <si>
+    <t>conv_k1p5</t>
+  </si>
+  <si>
+    <t>conv_k3</t>
+  </si>
+  <si>
+    <t>conv_k5</t>
+  </si>
+  <si>
+    <t>conv_k7</t>
+  </si>
+  <si>
+    <t>conv_k10</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>2024-07</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>assistant</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>DeepSeek</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Grok</t>
+  </si>
+  <si>
+    <t>Microsoft Copilot</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Perplexity</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>DeepSeek</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Grok</t>
+  </si>
+  <si>
+    <t>Microsoft Copilot</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Perplexity</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>DeepSeek</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Grok</t>
+  </si>
+  <si>
+    <t>Microsoft Copilot</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Perplexity</t>
+  </si>
+  <si>
+    <t>unique_users</t>
+  </si>
+  <si>
+    <t>share_ww_pct</t>
+  </si>
+  <si>
+    <t>msgs_per_user</t>
+  </si>
+  <si>
+    <t>messages</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>2024-07</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>assistant</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>DeepSeek</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Grok</t>
+  </si>
+  <si>
+    <t>Microsoft Copilot</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Perplexity</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>DeepSeek</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Grok</t>
+  </si>
+  <si>
+    <t>Microsoft Copilot</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Perplexity</t>
+  </si>
+  <si>
+    <t>ChatGPT</t>
+  </si>
+  <si>
+    <t>Claude</t>
+  </si>
+  <si>
+    <t>DeepSeek</t>
+  </si>
+  <si>
+    <t>Google Gemini</t>
+  </si>
+  <si>
+    <t>Grok</t>
+  </si>
+  <si>
+    <t>Microsoft Copilot</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Perplexity</t>
+  </si>
+  <si>
+    <t>unique_users</t>
+  </si>
+  <si>
+    <t>share_ww_pct</t>
+  </si>
+  <si>
+    <t>msgs_per_user</t>
+  </si>
+  <si>
+    <t>messages</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>market</t>
+  </si>
+  <si>
+    <t>Argentina</t>
+  </si>
+  <si>
+    <t>Australia</t>
+  </si>
+  <si>
+    <t>Brazil</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Indonesia</t>
+  </si>
+  <si>
+    <t>Italy</t>
+  </si>
+  <si>
+    <t>Japan</t>
+  </si>
+  <si>
+    <t>Mexico</t>
+  </si>
+  <si>
+    <t>South Korea</t>
+  </si>
+  <si>
+    <t>Spain</t>
+  </si>
+  <si>
+    <t>Taiwan</t>
+  </si>
+  <si>
+    <t>Turkey</t>
+  </si>
+  <si>
+    <t>United Kingdom</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>Vietnam</t>
+  </si>
+  <si>
+    <t>Other 7 markets (residual)</t>
+  </si>
+  <si>
+    <t>iso2</t>
+  </si>
+  <si>
+    <t>AR</t>
+  </si>
+  <si>
+    <t>AU</t>
+  </si>
+  <si>
+    <t>BR</t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t>FR</t>
+  </si>
+  <si>
+    <t>DE</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>JP</t>
+  </si>
+  <si>
+    <t>MX</t>
+  </si>
+  <si>
+    <t>KR</t>
+  </si>
+  <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>TW</t>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+  <si>
+    <t>GB</t>
+  </si>
+  <si>
+    <t>US</t>
+  </si>
+  <si>
+    <t>VN</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>residual</t>
+  </si>
+  <si>
+    <t>all_users</t>
+  </si>
+  <si>
+    <t>messages</t>
+  </si>
+  <si>
+    <t>work_share</t>
+  </si>
+  <si>
+    <t>work_share_src</t>
+  </si>
+  <si>
+    <t>Signals 국가별</t>
+  </si>
+  <si>
+    <t>Signals 전 세계(residual)</t>
+  </si>
+  <si>
+    <t>work_messages</t>
+  </si>
+  <si>
+    <t>nonwork_messages</t>
+  </si>
+  <si>
+    <t>conv_k1p5</t>
+  </si>
+  <si>
+    <t>conv_k3</t>
+  </si>
+  <si>
+    <t>conv_k5</t>
+  </si>
+  <si>
+    <t>conv_k7</t>
+  </si>
+  <si>
+    <t>conv_k10</t>
+  </si>
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>2024-07</t>
+  </si>
+  <si>
+    <t>2024-08</t>
+  </si>
+  <si>
+    <t>2024-09</t>
+  </si>
+  <si>
+    <t>2024-10</t>
+  </si>
+  <si>
+    <t>2024-11</t>
+  </si>
+  <si>
+    <t>2024-12</t>
+  </si>
+  <si>
+    <t>2025-01</t>
+  </si>
+  <si>
+    <t>2025-02</t>
+  </si>
+  <si>
+    <t>2025-03</t>
+  </si>
+  <si>
+    <t>2025-04</t>
+  </si>
+  <si>
+    <t>2025-05</t>
+  </si>
+  <si>
+    <t>2025-06</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>market</t>
+  </si>
+  <si>
+    <t>Worldwide</t>
+  </si>
+  <si>
+    <t>worldwide_users</t>
+  </si>
+  <si>
+    <t>msgs_per_user</t>
+  </si>
+  <si>
+    <t>messages</t>
+  </si>
+  <si>
+    <t>work_share_implied</t>
+  </si>
+  <si>
+    <t>work_messages</t>
+  </si>
+  <si>
+    <t>nonwork_messages</t>
+  </si>
+  <si>
+    <t>work_share_global</t>
+  </si>
+  <si>
+    <t>work_messages_global</t>
+  </si>
+  <si>
+    <t>conv_k1p5</t>
+  </si>
+  <si>
+    <t>conv_k3</t>
+  </si>
+  <si>
+    <t>conv_k5</t>
+  </si>
+  <si>
+    <t>conv_k7</t>
+  </si>
+  <si>
+    <t>conv_k10</t>
+  </si>
   <si>
     <t>month</t>
   </si>
@@ -449,502 +1316,502 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>289</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>293</v>
       </c>
       <c r="C1" t="s">
-        <v>29</v>
+        <v>318</v>
       </c>
       <c r="D1" t="s">
-        <v>30</v>
+        <v>319</v>
       </c>
       <c r="E1" t="s">
-        <v>31</v>
+        <v>320</v>
       </c>
       <c r="F1" t="s">
-        <v>32</v>
+        <v>321</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>290</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>294</v>
       </c>
       <c r="C2" s="1">
-        <v>502000000</v>
+        <v>461570000</v>
       </c>
       <c r="D2" s="1">
-        <v>71.056706649039313</v>
+        <v>71.327368374758066</v>
       </c>
       <c r="E2" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F2" s="1">
-        <v>40258120149.468239</v>
+        <v>24809261751.10104</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>290</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>295</v>
       </c>
       <c r="C3" s="1">
-        <v>24600000</v>
+        <v>22503000</v>
       </c>
       <c r="D3" s="1">
-        <v>3.4820617202517279</v>
+        <v>3.4774352114244449</v>
       </c>
       <c r="E3" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F3" s="1">
-        <v>1972808278.2408738</v>
+        <v>1209530119.342736</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>1</v>
+        <v>290</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>296</v>
       </c>
       <c r="C4" s="1">
-        <v>388000</v>
+        <v>216940</v>
       </c>
       <c r="D4" s="1">
-        <v>0.05492032306738498</v>
+        <v>0.033524187653487046</v>
       </c>
       <c r="E4" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F4" s="1">
-        <v>31115837.884449556</v>
+        <v>11660465.89744537</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>1</v>
+        <v>290</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>297</v>
       </c>
       <c r="C5" s="1">
-        <v>88200000</v>
+        <v>79498000</v>
       </c>
       <c r="D5" s="1">
-        <v>12.484465192122048</v>
+        <v>12.284990642928522</v>
       </c>
       <c r="E5" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F5" s="1">
-        <v>7073239436.6197186</v>
+        <v>4272995841.7770443</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>1</v>
+        <v>290</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>298</v>
       </c>
       <c r="C6" s="1">
-        <v>1190000</v>
+        <v>1197920</v>
       </c>
       <c r="D6" s="1">
-        <v>0.16844119703656729</v>
+        <v>0.18511705943516735</v>
       </c>
       <c r="E6" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F6" s="1">
-        <v>95432595.573440641</v>
+        <v>64387873.641872212</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>1</v>
+        <v>290</v>
       </c>
       <c r="B7" t="s">
-        <v>10</v>
+        <v>299</v>
       </c>
       <c r="C7" s="1">
-        <v>22600000</v>
+        <v>20641000</v>
       </c>
       <c r="D7" s="1">
-        <v>3.198967271450774</v>
+        <v>3.1896964937569194</v>
       </c>
       <c r="E7" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F7" s="1">
-        <v>1812417361.3107214</v>
+        <v>1109448126.6210468</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>1</v>
+        <v>290</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>300</v>
       </c>
       <c r="C8" s="1">
-        <v>44900000</v>
+        <v>41000000</v>
       </c>
       <c r="D8" s="1">
-        <v>6.3554703755814055</v>
+        <v>6.3358149432698854</v>
       </c>
       <c r="E8" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F8" s="1">
-        <v>3600776085.0819201</v>
+        <v>2203738830.0694208</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>1</v>
+        <v>290</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>301</v>
       </c>
       <c r="C9" s="1">
-        <v>22600000</v>
+        <v>20488000</v>
       </c>
       <c r="D9" s="1">
-        <v>3.198967271450774</v>
+        <v>3.1660530867734979</v>
       </c>
       <c r="E9" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F9" s="1">
-        <v>1812417361.3107214</v>
+        <v>1101224418.3039584</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>2</v>
+        <v>291</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>302</v>
       </c>
       <c r="C10" s="1">
-        <v>994000000</v>
+        <v>904770000</v>
       </c>
       <c r="D10" s="1">
-        <v>58.00315107661784</v>
+        <v>58.165750885726354</v>
       </c>
       <c r="E10" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F10" s="1">
-        <v>79714285714.285721</v>
+        <v>48631141006.875854</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>2</v>
+        <v>291</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>303</v>
       </c>
       <c r="C11" s="1">
-        <v>49000000</v>
+        <v>44792000</v>
       </c>
       <c r="D11" s="1">
-        <v>2.8593102643403161</v>
+        <v>2.8795830030543175</v>
       </c>
       <c r="E11" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F11" s="1">
-        <v>3929577464.7887325</v>
+        <v>2407557796.987061</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2</v>
+        <v>291</v>
       </c>
       <c r="B12" t="s">
-        <v>15</v>
+        <v>304</v>
       </c>
       <c r="C12" s="1">
-        <v>81900000</v>
+        <v>59245000</v>
       </c>
       <c r="D12" s="1">
-        <v>4.7791328703973859</v>
+        <v>3.8087358237174724</v>
       </c>
       <c r="E12" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F12" s="1">
-        <v>6568008048.2897387</v>
+        <v>3184402609.4503131</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2</v>
+        <v>291</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>305</v>
       </c>
       <c r="C13" s="1">
-        <v>331000000</v>
+        <v>308360000</v>
       </c>
       <c r="D13" s="1">
-        <v>19.314932601972341</v>
+        <v>19.823812618812049</v>
       </c>
       <c r="E13" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F13" s="1">
-        <v>26544696751.940212</v>
+        <v>16574265991.224552</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2</v>
+        <v>291</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
+        <v>306</v>
       </c>
       <c r="C14" s="1">
-        <v>60100000</v>
+        <v>54088000</v>
       </c>
       <c r="D14" s="1">
-        <v>3.5070315691194489</v>
+        <v>3.4772031940793431</v>
       </c>
       <c r="E14" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F14" s="1">
-        <v>4819747053.7510777</v>
+        <v>2907215264.4096303</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>2</v>
+        <v>291</v>
       </c>
       <c r="B15" t="s">
-        <v>18</v>
+        <v>307</v>
       </c>
       <c r="C15" s="1">
-        <v>39700000</v>
+        <v>36903000</v>
       </c>
       <c r="D15" s="1">
-        <v>2.3166248468226645</v>
+        <v>2.3724158680503993</v>
       </c>
       <c r="E15" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F15" s="1">
-        <v>3183759701.0635242</v>
+        <v>1983526196.2451668</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2</v>
+        <v>291</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>308</v>
       </c>
       <c r="C16" s="1">
-        <v>58600000</v>
+        <v>54400000</v>
       </c>
       <c r="D16" s="1">
-        <v>3.4195016630682149</v>
+        <v>3.4972610146042791</v>
       </c>
       <c r="E16" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F16" s="1">
-        <v>4699453866.0534639</v>
+        <v>2923985179.409183</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>2</v>
+        <v>291</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>309</v>
       </c>
       <c r="C17" s="1">
-        <v>99400000</v>
+        <v>92945000</v>
       </c>
       <c r="D17" s="1">
-        <v>5.8003151076617847</v>
+        <v>5.9752375919557856</v>
       </c>
       <c r="E17" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F17" s="1">
-        <v>7971428571.4285717</v>
+        <v>4995768428.312252</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>3</v>
+        <v>292</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>310</v>
       </c>
       <c r="C18" s="1">
-        <v>1110000000</v>
+        <v>1010840000</v>
       </c>
       <c r="D18" s="1">
-        <v>46.461010422334766</v>
+        <v>46.931795125842157</v>
       </c>
       <c r="E18" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F18" s="1">
-        <v>89016958896.234558</v>
+        <v>54332374609.448135</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>3</v>
+        <v>292</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
+        <v>311</v>
       </c>
       <c r="C19" s="1">
-        <v>245000000</v>
+        <v>222120000</v>
       </c>
       <c r="D19" s="1">
-        <v>10.254907705830647</v>
+        <v>10.312700658216988</v>
       </c>
       <c r="E19" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F19" s="1">
-        <v>19647887323.943661</v>
+        <v>11938889486.219994</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>3</v>
+        <v>292</v>
       </c>
       <c r="B20" t="s">
-        <v>23</v>
+        <v>312</v>
       </c>
       <c r="C20" s="1">
-        <v>75800000</v>
+        <v>46656000</v>
       </c>
       <c r="D20" s="1">
-        <v>3.1727428738855639</v>
+        <v>2.1661685661343948</v>
       </c>
       <c r="E20" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F20" s="1">
-        <v>6078815751.6527739</v>
+        <v>2507747289.1638756</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>3</v>
+        <v>292</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>313</v>
       </c>
       <c r="C21" s="1">
-        <v>662000000</v>
+        <v>604630000</v>
       </c>
       <c r="D21" s="1">
-        <v>27.709179188815874</v>
+        <v>28.072070047621722</v>
       </c>
       <c r="E21" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F21" s="1">
-        <v>53089393503.880424</v>
+        <v>32498697776.216438</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>3</v>
+        <v>292</v>
       </c>
       <c r="B22" t="s">
-        <v>25</v>
+        <v>314</v>
       </c>
       <c r="C22" s="1">
-        <v>78100000</v>
+        <v>68207000</v>
       </c>
       <c r="D22" s="1">
-        <v>3.269013436021933</v>
+        <v>3.1667493867954533</v>
       </c>
       <c r="E22" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F22" s="1">
-        <v>6263265306.1224489</v>
+        <v>3666107667.866951</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>3</v>
+        <v>292</v>
       </c>
       <c r="B23" t="s">
-        <v>26</v>
+        <v>315</v>
       </c>
       <c r="C23" s="1">
-        <v>38500000</v>
+        <v>35572000</v>
       </c>
       <c r="D23" s="1">
-        <v>1.6114854966305305</v>
+        <v>1.6515549604452309</v>
       </c>
       <c r="E23" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F23" s="1">
-        <v>3087525150.9054327</v>
+        <v>1911985308.8592546</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>3</v>
+        <v>292</v>
       </c>
       <c r="B24" t="s">
-        <v>27</v>
+        <v>316</v>
       </c>
       <c r="C24" s="1">
-        <v>111800000</v>
+        <v>104200000</v>
       </c>
       <c r="D24" s="1">
-        <v>4.6795864551504751</v>
+        <v>4.8378507499829375</v>
       </c>
       <c r="E24" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F24" s="1">
-        <v>8965852256.3955154</v>
+        <v>5600721612.0300894</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>3</v>
+        <v>292</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>317</v>
       </c>
       <c r="C25" s="1">
-        <v>67900000</v>
+        <v>61624000</v>
       </c>
       <c r="D25" s="1">
-        <v>2.8420744213302078</v>
+        <v>2.8611105049611183</v>
       </c>
       <c r="E25" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="F25" s="1">
-        <v>5445271629.7786722</v>
+        <v>3312273211.3219023</v>
       </c>
     </row>
   </sheetData>
@@ -958,60 +1825,60 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>322</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>324</v>
       </c>
       <c r="C1" t="s">
-        <v>55</v>
+        <v>344</v>
       </c>
       <c r="D1" t="s">
-        <v>75</v>
+        <v>364</v>
       </c>
       <c r="E1" t="s">
-        <v>76</v>
+        <v>365</v>
       </c>
       <c r="F1" t="s">
-        <v>77</v>
+        <v>366</v>
       </c>
       <c r="G1" t="s">
-        <v>78</v>
+        <v>367</v>
       </c>
       <c r="H1" t="s">
-        <v>79</v>
+        <v>368</v>
       </c>
       <c r="I1" t="s">
-        <v>82</v>
+        <v>371</v>
       </c>
       <c r="J1" t="s">
-        <v>83</v>
+        <v>372</v>
       </c>
       <c r="K1" t="s">
-        <v>84</v>
+        <v>373</v>
       </c>
       <c r="L1" t="s">
-        <v>85</v>
+        <v>374</v>
       </c>
       <c r="M1" t="s">
-        <v>86</v>
+        <v>375</v>
       </c>
       <c r="N1" t="s">
-        <v>87</v>
+        <v>376</v>
       </c>
       <c r="O1" t="s">
-        <v>88</v>
+        <v>377</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>325</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>345</v>
       </c>
       <c r="D2" s="1">
         <v>0</v>
@@ -1020,45 +1887,45 @@
         <v>38419000</v>
       </c>
       <c r="F2" s="1">
-        <v>3081029318.7697616</v>
+        <v>2065010783.2301726</v>
       </c>
       <c r="G2" s="1">
         <v>0.29100000858306885</v>
       </c>
       <c r="H2" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I2" s="1">
-        <v>896579558.20668733</v>
+        <v>600918155.64410996</v>
       </c>
       <c r="J2" s="1">
-        <v>2184449760.5630741</v>
+        <v>1464092627.5860627</v>
       </c>
       <c r="K2" s="1">
-        <v>597719705.47112489</v>
+        <v>400612103.76273996</v>
       </c>
       <c r="L2" s="1">
-        <v>298859852.73556244</v>
+        <v>200306051.88136998</v>
       </c>
       <c r="M2" s="1">
-        <v>179315911.64133745</v>
+        <v>120183631.128822</v>
       </c>
       <c r="N2" s="1">
-        <v>128082794.02952676</v>
+        <v>85845450.80630143</v>
       </c>
       <c r="O2" s="1">
-        <v>89657955.820668727</v>
+        <v>60091815.564410999</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B3" t="s">
-        <v>37</v>
+        <v>326</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>346</v>
       </c>
       <c r="D3" s="1">
         <v>0</v>
@@ -1067,45 +1934,45 @@
         <v>26118000</v>
       </c>
       <c r="F3" s="1">
-        <v>2094544984.1908596</v>
+        <v>1403835384.4817839</v>
       </c>
       <c r="G3" s="1">
         <v>0.3970000147819519</v>
       </c>
       <c r="H3" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I3" s="1">
-        <v>831534389.68523443</v>
+        <v>557322668.39069533</v>
       </c>
       <c r="J3" s="1">
-        <v>1263010594.5056252</v>
+        <v>846512716.09108853</v>
       </c>
       <c r="K3" s="1">
-        <v>554356259.79015625</v>
+        <v>371548445.59379691</v>
       </c>
       <c r="L3" s="1">
-        <v>277178129.89507812</v>
+        <v>185774222.79689845</v>
       </c>
       <c r="M3" s="1">
-        <v>166306877.93704689</v>
+        <v>111464533.67813906</v>
       </c>
       <c r="N3" s="1">
-        <v>118790627.09789063</v>
+        <v>79617524.055813625</v>
       </c>
       <c r="O3" s="1">
-        <v>83153438.968523443</v>
+        <v>55732266.83906953</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>327</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>347</v>
       </c>
       <c r="D4" s="1">
         <v>0</v>
@@ -1114,45 +1981,45 @@
         <v>209550000</v>
       </c>
       <c r="F4" s="1">
-        <v>16804958321.356712</v>
+        <v>11263255410.757248</v>
       </c>
       <c r="G4" s="1">
         <v>0.35400000214576721</v>
       </c>
       <c r="H4" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I4" s="1">
-        <v>5948955281.8198051</v>
+        <v>3987192439.5763898</v>
       </c>
       <c r="J4" s="1">
-        <v>10856003039.536907</v>
+        <v>7276062971.1808586</v>
       </c>
       <c r="K4" s="1">
-        <v>3965970187.8798699</v>
+        <v>2658128293.0509267</v>
       </c>
       <c r="L4" s="1">
-        <v>1982985093.939935</v>
+        <v>1329064146.5254633</v>
       </c>
       <c r="M4" s="1">
-        <v>1189791056.363961</v>
+        <v>797438487.91527796</v>
       </c>
       <c r="N4" s="1">
-        <v>849850754.54568648</v>
+        <v>569598919.93948424</v>
       </c>
       <c r="O4" s="1">
-        <v>594895528.18198049</v>
+        <v>398719243.95763898</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>328</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>348</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
@@ -1161,45 +2028,45 @@
         <v>39835000</v>
       </c>
       <c r="F5" s="1">
-        <v>3194586087.9563093</v>
+        <v>2141120397.4589117</v>
       </c>
       <c r="G5" s="1">
         <v>0.32899999618530273</v>
       </c>
       <c r="H5" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I5" s="1">
-        <v>1051018810.7512469</v>
+        <v>704428602.59625578</v>
       </c>
       <c r="J5" s="1">
-        <v>2143567277.2050624</v>
+        <v>1436691794.8626559</v>
       </c>
       <c r="K5" s="1">
-        <v>700679207.16749799</v>
+        <v>469619068.39750385</v>
       </c>
       <c r="L5" s="1">
-        <v>350339603.583749</v>
+        <v>234809534.19875193</v>
       </c>
       <c r="M5" s="1">
-        <v>210203762.15024939</v>
+        <v>140885720.51925117</v>
       </c>
       <c r="N5" s="1">
-        <v>150145544.39303526</v>
+        <v>100632657.51375082</v>
       </c>
       <c r="O5" s="1">
-        <v>105101881.0751247</v>
+        <v>70442860.259625584</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>329</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>349</v>
       </c>
       <c r="D6" s="1">
         <v>0</v>
@@ -1208,45 +2075,45 @@
         <v>59780000</v>
       </c>
       <c r="F6" s="1">
-        <v>4794084507.0422535</v>
+        <v>3213158713.696341</v>
       </c>
       <c r="G6" s="1">
         <v>0.25499999523162842</v>
       </c>
       <c r="H6" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I6" s="1">
-        <v>1222491526.4357984</v>
+        <v>819355456.67103231</v>
       </c>
       <c r="J6" s="1">
-        <v>3571592980.6064548</v>
+        <v>2393803257.0253086</v>
       </c>
       <c r="K6" s="1">
-        <v>814994350.95719898</v>
+        <v>546236971.11402154</v>
       </c>
       <c r="L6" s="1">
-        <v>407497175.47859949</v>
+        <v>273118485.55701077</v>
       </c>
       <c r="M6" s="1">
-        <v>244498305.28715968</v>
+        <v>163871091.33420646</v>
       </c>
       <c r="N6" s="1">
-        <v>174641646.6336855</v>
+        <v>117050779.52443318</v>
       </c>
       <c r="O6" s="1">
-        <v>122249152.64357984</v>
+        <v>81935545.667103231</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>330</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>350</v>
       </c>
       <c r="D7" s="1">
         <v>0</v>
@@ -1255,45 +2122,45 @@
         <v>69110000</v>
       </c>
       <c r="F7" s="1">
-        <v>5542308134.5214138</v>
+        <v>3714643671.856041</v>
       </c>
       <c r="G7" s="1">
         <v>0.26100000739097595</v>
       </c>
       <c r="H7" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I7" s="1">
-        <v>1446542464.0731552</v>
+        <v>969522025.80926871</v>
       </c>
       <c r="J7" s="1">
-        <v>4095765670.4482584</v>
+        <v>2745121646.046772</v>
       </c>
       <c r="K7" s="1">
-        <v>964361642.71543682</v>
+        <v>646348017.20617914</v>
       </c>
       <c r="L7" s="1">
-        <v>482180821.35771841</v>
+        <v>323174008.60308957</v>
       </c>
       <c r="M7" s="1">
-        <v>289308492.81463104</v>
+        <v>193904405.16185373</v>
       </c>
       <c r="N7" s="1">
-        <v>206648923.43902215</v>
+        <v>138503146.54418126</v>
       </c>
       <c r="O7" s="1">
-        <v>144654246.40731552</v>
+        <v>96952202.580926865</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>331</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>351</v>
       </c>
       <c r="D8" s="1">
         <v>0</v>
@@ -1302,45 +2169,45 @@
         <v>724030000</v>
       </c>
       <c r="F8" s="1">
-        <v>58063917792.469101</v>
+        <v>38916415247.199097</v>
       </c>
       <c r="G8" s="1">
         <v>0.33199998736381531</v>
       </c>
       <c r="H8" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I8" s="1">
-        <v>19277219973.393353</v>
+        <v>12920249370.31509</v>
       </c>
       <c r="J8" s="1">
-        <v>38786697819.075745</v>
+        <v>25996165876.884007</v>
       </c>
       <c r="K8" s="1">
-        <v>12851479982.262236</v>
+        <v>8613499580.2100601</v>
       </c>
       <c r="L8" s="1">
-        <v>6425739991.1311178</v>
+        <v>4306749790.1050301</v>
       </c>
       <c r="M8" s="1">
-        <v>3855443994.6786704</v>
+        <v>2584049874.0630178</v>
       </c>
       <c r="N8" s="1">
-        <v>2753888567.6276217</v>
+        <v>1845749910.045013</v>
       </c>
       <c r="O8" s="1">
-        <v>1927721997.3393352</v>
+        <v>1292024937.0315089</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B9" t="s">
-        <v>43</v>
+        <v>332</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>352</v>
       </c>
       <c r="D9" s="1">
         <v>0</v>
@@ -1349,45 +2216,45 @@
         <v>126909000</v>
       </c>
       <c r="F9" s="1">
-        <v>10177525438.344353</v>
+        <v>6821324175.2507353</v>
       </c>
       <c r="G9" s="1">
         <v>0.40799999237060547</v>
       </c>
       <c r="H9" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I9" s="1">
-        <v>4152430301.1961389</v>
+        <v>2783100211.4597268</v>
       </c>
       <c r="J9" s="1">
-        <v>6025095137.1482143</v>
+        <v>4038223963.7910085</v>
       </c>
       <c r="K9" s="1">
-        <v>2768286867.4640927</v>
+        <v>1855400140.9731512</v>
       </c>
       <c r="L9" s="1">
-        <v>1384143433.7320464</v>
+        <v>927700070.4865756</v>
       </c>
       <c r="M9" s="1">
-        <v>830486060.23922777</v>
+        <v>556620042.29194534</v>
       </c>
       <c r="N9" s="1">
-        <v>593204328.74230552</v>
+        <v>397585744.49424666</v>
       </c>
       <c r="O9" s="1">
-        <v>415243030.11961389</v>
+        <v>278310021.14597267</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>333</v>
       </c>
       <c r="C10" t="s">
-        <v>64</v>
+        <v>353</v>
       </c>
       <c r="D10" s="1">
         <v>0</v>
@@ -1396,45 +2263,45 @@
         <v>47617000</v>
       </c>
       <c r="F10" s="1">
-        <v>3818667145.7315321</v>
+        <v>2559400777.3516002</v>
       </c>
       <c r="G10" s="1">
         <v>0.30500000715255737</v>
       </c>
       <c r="H10" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I10" s="1">
-        <v>1164693506.7613533</v>
+        <v>780617255.39849901</v>
       </c>
       <c r="J10" s="1">
-        <v>2653973638.9701786</v>
+        <v>1778783521.9531012</v>
       </c>
       <c r="K10" s="1">
-        <v>776462337.84090221</v>
+        <v>520411503.59899932</v>
       </c>
       <c r="L10" s="1">
-        <v>388231168.9204511</v>
+        <v>260205751.79949966</v>
       </c>
       <c r="M10" s="1">
-        <v>232938701.35227066</v>
+        <v>156123451.07969981</v>
       </c>
       <c r="N10" s="1">
-        <v>166384786.68019333</v>
+        <v>111516750.77121414</v>
       </c>
       <c r="O10" s="1">
-        <v>116469350.67613533</v>
+        <v>78061725.539849907</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>334</v>
       </c>
       <c r="C11" t="s">
-        <v>65</v>
+        <v>354</v>
       </c>
       <c r="D11" s="1">
         <v>0</v>
@@ -1443,45 +2310,45 @@
         <v>101730000</v>
       </c>
       <c r="F11" s="1">
-        <v>8158283989.6521988</v>
+        <v>5467959784.9502974</v>
       </c>
       <c r="G11" s="1">
         <v>0.27799999713897705</v>
       </c>
       <c r="H11" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I11" s="1">
-        <v>2268002925.7822738</v>
+        <v>1520092804.5722241</v>
       </c>
       <c r="J11" s="1">
-        <v>5890281063.8699245</v>
+        <v>3947866980.3780732</v>
       </c>
       <c r="K11" s="1">
-        <v>1512001950.5215158</v>
+        <v>1013395203.0481495</v>
       </c>
       <c r="L11" s="1">
-        <v>756000975.26075792</v>
+        <v>506697601.52407473</v>
       </c>
       <c r="M11" s="1">
-        <v>453600585.15645474</v>
+        <v>304018560.9144448</v>
       </c>
       <c r="N11" s="1">
-        <v>324000417.96889627</v>
+        <v>217156114.93888918</v>
       </c>
       <c r="O11" s="1">
-        <v>226800292.57822737</v>
+        <v>152009280.4572224</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>335</v>
       </c>
       <c r="C12" t="s">
-        <v>66</v>
+        <v>355</v>
       </c>
       <c r="D12" s="1">
         <v>0</v>
@@ -1490,45 +2357,45 @@
         <v>92580000</v>
       </c>
       <c r="F12" s="1">
-        <v>7424495544.6967516</v>
+        <v>4976149777.7518778</v>
       </c>
       <c r="G12" s="1">
         <v>0.29100000858306885</v>
       </c>
       <c r="H12" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I12" s="1">
-        <v>2160528267.2317109</v>
+        <v>1448059628.0364325</v>
       </c>
       <c r="J12" s="1">
-        <v>5263967277.4650402</v>
+        <v>3528090149.7154455</v>
       </c>
       <c r="K12" s="1">
-        <v>1440352178.154474</v>
+        <v>965373085.35762167</v>
       </c>
       <c r="L12" s="1">
-        <v>720176089.07723701</v>
+        <v>482686542.67881083</v>
       </c>
       <c r="M12" s="1">
-        <v>432105653.44634217</v>
+        <v>289611925.60728651</v>
       </c>
       <c r="N12" s="1">
-        <v>308646895.31881583</v>
+        <v>206865661.14806178</v>
       </c>
       <c r="O12" s="1">
-        <v>216052826.72317109</v>
+        <v>144805962.80364326</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>336</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>356</v>
       </c>
       <c r="D13" s="1">
         <v>0</v>
@@ -1537,45 +2404,45 @@
         <v>60970000</v>
       </c>
       <c r="F13" s="1">
-        <v>4889517102.615694</v>
+        <v>3277120889.4959168</v>
       </c>
       <c r="G13" s="1">
         <v>0.31700000166893005</v>
       </c>
       <c r="H13" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I13" s="1">
-        <v>1549976929.6894372</v>
+        <v>1038847327.4394912</v>
       </c>
       <c r="J13" s="1">
-        <v>3339540172.9262571</v>
+        <v>2238273562.0564256</v>
       </c>
       <c r="K13" s="1">
-        <v>1033317953.1262914</v>
+        <v>692564884.95966077</v>
       </c>
       <c r="L13" s="1">
-        <v>516658976.5631457</v>
+        <v>346282442.47983038</v>
       </c>
       <c r="M13" s="1">
-        <v>309995385.93788743</v>
+        <v>207769465.48789823</v>
       </c>
       <c r="N13" s="1">
-        <v>221425275.66991958</v>
+        <v>148406761.06278446</v>
       </c>
       <c r="O13" s="1">
-        <v>154997692.96894372</v>
+        <v>103884732.74394912</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B14" t="s">
-        <v>48</v>
+        <v>337</v>
       </c>
       <c r="C14" t="s">
-        <v>68</v>
+        <v>357</v>
       </c>
       <c r="D14" s="1">
         <v>0</v>
@@ -1584,45 +2451,45 @@
         <v>53340000</v>
       </c>
       <c r="F14" s="1">
-        <v>4277625754.527163</v>
+        <v>2867010468.1927538</v>
       </c>
       <c r="G14" s="1">
         <v>0.29800000786781311</v>
       </c>
       <c r="H14" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I14" s="1">
-        <v>1274732508.5046546</v>
+        <v>854369142.07854319</v>
       </c>
       <c r="J14" s="1">
-        <v>3002893246.0225086</v>
+        <v>2012641326.1142106</v>
       </c>
       <c r="K14" s="1">
-        <v>849821672.33643639</v>
+        <v>569579428.05236208</v>
       </c>
       <c r="L14" s="1">
-        <v>424910836.1682182</v>
+        <v>284789714.02618104</v>
       </c>
       <c r="M14" s="1">
-        <v>254946501.70093092</v>
+        <v>170873828.41570863</v>
       </c>
       <c r="N14" s="1">
-        <v>182104644.07209352</v>
+        <v>122052734.58264902</v>
       </c>
       <c r="O14" s="1">
-        <v>127473250.85046546</v>
+        <v>85436914.207854316</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>338</v>
       </c>
       <c r="C15" t="s">
-        <v>69</v>
+        <v>358</v>
       </c>
       <c r="D15" s="1">
         <v>0</v>
@@ -1631,45 +2498,45 @@
         <v>20672000</v>
       </c>
       <c r="F15" s="1">
-        <v>1657800517.3900547</v>
+        <v>1111114368.1754894</v>
       </c>
       <c r="G15" s="1">
         <v>0.33500000834465027</v>
       </c>
       <c r="H15" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I15" s="1">
-        <v>555363187.15943384</v>
+        <v>372223322.61064976</v>
       </c>
       <c r="J15" s="1">
-        <v>1102437330.2306209</v>
+        <v>738891045.5648396</v>
       </c>
       <c r="K15" s="1">
-        <v>370242124.77295589</v>
+        <v>248148881.74043319</v>
       </c>
       <c r="L15" s="1">
-        <v>185121062.38647795</v>
+        <v>124074440.87021659</v>
       </c>
       <c r="M15" s="1">
-        <v>111072637.43188676</v>
+        <v>74444664.522129953</v>
       </c>
       <c r="N15" s="1">
-        <v>79337598.16563341</v>
+        <v>53174760.372949965</v>
       </c>
       <c r="O15" s="1">
-        <v>55536318.715943381</v>
+        <v>37222332.261064976</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>339</v>
       </c>
       <c r="C16" t="s">
-        <v>70</v>
+        <v>359</v>
       </c>
       <c r="D16" s="1">
         <v>0</v>
@@ -1678,45 +2545,45 @@
         <v>74937000</v>
       </c>
       <c r="F16" s="1">
-        <v>6009607070.9974127</v>
+        <v>4027843334.3637118</v>
       </c>
       <c r="G16" s="1">
         <v>0.18600000441074371</v>
       </c>
       <c r="H16" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I16" s="1">
-        <v>1117786941.7123554</v>
+        <v>749178877.95743501</v>
       </c>
       <c r="J16" s="1">
-        <v>4891820129.2850571</v>
+        <v>3278664456.4062767</v>
       </c>
       <c r="K16" s="1">
-        <v>745191294.47490358</v>
+        <v>499452585.30495667</v>
       </c>
       <c r="L16" s="1">
-        <v>372595647.23745179</v>
+        <v>249726292.65247834</v>
       </c>
       <c r="M16" s="1">
-        <v>223557388.34247106</v>
+        <v>149835775.59148699</v>
       </c>
       <c r="N16" s="1">
-        <v>159683848.81605077</v>
+        <v>107025553.99391928</v>
       </c>
       <c r="O16" s="1">
-        <v>111778694.17123553</v>
+        <v>74917887.795743495</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B17" t="s">
-        <v>51</v>
+        <v>340</v>
       </c>
       <c r="C17" t="s">
-        <v>71</v>
+        <v>360</v>
       </c>
       <c r="D17" s="1">
         <v>0</v>
@@ -1725,45 +2592,45 @@
         <v>56300000</v>
       </c>
       <c r="F17" s="1">
-        <v>4515004311.5837889</v>
+        <v>3026109661.7782536</v>
       </c>
       <c r="G17" s="1">
         <v>0.32600000500679016</v>
       </c>
       <c r="H17" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I17" s="1">
-        <v>1471891428.1819944</v>
+        <v>986511764.89080679</v>
       </c>
       <c r="J17" s="1">
-        <v>3043112883.4017944</v>
+        <v>2039597896.8874469</v>
       </c>
       <c r="K17" s="1">
-        <v>981260952.12132967</v>
+        <v>657674509.92720449</v>
       </c>
       <c r="L17" s="1">
-        <v>490630476.06066483</v>
+        <v>328837254.96360224</v>
       </c>
       <c r="M17" s="1">
-        <v>294378285.63639891</v>
+        <v>197302352.97816136</v>
       </c>
       <c r="N17" s="1">
-        <v>210270204.02599922</v>
+        <v>140930252.12725812</v>
       </c>
       <c r="O17" s="1">
-        <v>147189142.81819946</v>
+        <v>98651176.489080682</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B18" t="s">
-        <v>52</v>
+        <v>341</v>
       </c>
       <c r="C18" t="s">
-        <v>72</v>
+        <v>361</v>
       </c>
       <c r="D18" s="1">
         <v>0</v>
@@ -1772,45 +2639,45 @@
         <v>293620000</v>
       </c>
       <c r="F18" s="1">
-        <v>23546990514.515667</v>
+        <v>15781995006.950813</v>
       </c>
       <c r="G18" s="1">
         <v>0.32100000977516174</v>
       </c>
       <c r="H18" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I18" s="1">
-        <v>7558584185.3351698</v>
+        <v>5066020551.5027647</v>
       </c>
       <c r="J18" s="1">
-        <v>15988406329.180496</v>
+        <v>10715974455.448048</v>
       </c>
       <c r="K18" s="1">
-        <v>5039056123.5567799</v>
+        <v>3377347034.3351765</v>
       </c>
       <c r="L18" s="1">
-        <v>2519528061.7783899</v>
+        <v>1688673517.1675882</v>
       </c>
       <c r="M18" s="1">
-        <v>1511716837.067034</v>
+        <v>1013204110.300553</v>
       </c>
       <c r="N18" s="1">
-        <v>1079797740.7621672</v>
+        <v>723717221.64325213</v>
       </c>
       <c r="O18" s="1">
-        <v>755858418.533517</v>
+        <v>506602055.15027648</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>342</v>
       </c>
       <c r="C19" t="s">
-        <v>73</v>
+        <v>362</v>
       </c>
       <c r="D19" s="1">
         <v>0</v>
@@ -1819,45 +2686,45 @@
         <v>58332000</v>
       </c>
       <c r="F19" s="1">
-        <v>4677961483.184823</v>
+        <v>3135329108.1855965</v>
       </c>
       <c r="G19" s="1">
         <v>0.31799998879432678</v>
       </c>
       <c r="H19" t="s">
-        <v>80</v>
+        <v>369</v>
       </c>
       <c r="I19" s="1">
-        <v>1487591699.2330661</v>
+        <v>997034621.26954627</v>
       </c>
       <c r="J19" s="1">
-        <v>3190369783.951757</v>
+        <v>2138294486.9160502</v>
       </c>
       <c r="K19" s="1">
-        <v>991727799.48871076</v>
+        <v>664689747.51303089</v>
       </c>
       <c r="L19" s="1">
-        <v>495863899.74435538</v>
+        <v>332344873.75651544</v>
       </c>
       <c r="M19" s="1">
-        <v>297518339.84661323</v>
+        <v>199406924.25390926</v>
       </c>
       <c r="N19" s="1">
-        <v>212513099.89043802</v>
+        <v>142433517.3242209</v>
       </c>
       <c r="O19" s="1">
-        <v>148759169.92330661</v>
+        <v>99703462.12695463</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>34</v>
+        <v>323</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>343</v>
       </c>
       <c r="C20" t="s">
-        <v>74</v>
+        <v>363</v>
       </c>
       <c r="D20" s="1">
         <v>1</v>
@@ -1866,34 +2733,34 @@
         <v>235251000</v>
       </c>
       <c r="F20" s="1">
-        <v>18866061799.367634</v>
+        <v>12644677158.845398</v>
       </c>
       <c r="G20" s="1">
         <v>0.30500000715255737</v>
       </c>
       <c r="H20" t="s">
-        <v>81</v>
+        <v>370</v>
       </c>
       <c r="I20" s="1">
-        <v>5754148983.7477179</v>
+        <v>3856626623.8896251</v>
       </c>
       <c r="J20" s="1">
-        <v>13111912815.619915</v>
+        <v>8788050534.9557724</v>
       </c>
       <c r="K20" s="1">
-        <v>3836099322.4984784</v>
+        <v>2571084415.9264169</v>
       </c>
       <c r="L20" s="1">
-        <v>1918049661.2492392</v>
+        <v>1285542207.9632084</v>
       </c>
       <c r="M20" s="1">
-        <v>1150829796.7495437</v>
+        <v>771325324.77792501</v>
       </c>
       <c r="N20" s="1">
-        <v>822021283.39253116</v>
+        <v>550946660.55566072</v>
       </c>
       <c r="O20" s="1">
-        <v>575414898.37477183</v>
+        <v>385662662.38896251</v>
       </c>
     </row>
   </sheetData>
@@ -1907,1130 +2774,1130 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>89</v>
+        <v>378</v>
       </c>
       <c r="B1" t="s">
-        <v>113</v>
+        <v>402</v>
       </c>
       <c r="C1" t="s">
-        <v>115</v>
+        <v>404</v>
       </c>
       <c r="D1" t="s">
-        <v>116</v>
+        <v>405</v>
       </c>
       <c r="E1" t="s">
-        <v>117</v>
+        <v>406</v>
       </c>
       <c r="F1" t="s">
-        <v>118</v>
+        <v>407</v>
       </c>
       <c r="G1" t="s">
-        <v>119</v>
+        <v>408</v>
       </c>
       <c r="H1" t="s">
-        <v>120</v>
+        <v>409</v>
       </c>
       <c r="I1" t="s">
-        <v>121</v>
+        <v>410</v>
       </c>
       <c r="J1" t="s">
-        <v>122</v>
+        <v>411</v>
       </c>
       <c r="K1" t="s">
-        <v>123</v>
+        <v>412</v>
       </c>
       <c r="L1" t="s">
-        <v>124</v>
+        <v>413</v>
       </c>
       <c r="M1" t="s">
-        <v>125</v>
+        <v>414</v>
       </c>
       <c r="N1" t="s">
-        <v>126</v>
+        <v>415</v>
       </c>
       <c r="O1" t="s">
-        <v>127</v>
+        <v>416</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>379</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C2" s="1">
         <v>706478000</v>
       </c>
       <c r="D2" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E2" s="1">
-        <v>56656327105.490082</v>
+        <v>37973000029.019127</v>
       </c>
       <c r="F2" s="1">
-        <v>0.53845284854361009</v>
+        <v>0.53845284854361031</v>
       </c>
       <c r="G2" s="1">
-        <v>30506760717.969685</v>
+        <v>20446670033.371944</v>
       </c>
       <c r="H2" s="1">
-        <v>26149566387.520397</v>
+        <v>17526329995.647186</v>
       </c>
       <c r="I2" s="1">
         <v>0.5130000114440918</v>
       </c>
       <c r="J2" s="1">
-        <v>29064696453.49662</v>
+        <v>19480149449.453312</v>
       </c>
       <c r="K2" s="1">
-        <v>20337840478.646458</v>
+        <v>13631113355.581297</v>
       </c>
       <c r="L2" s="1">
-        <v>10168920239.323229</v>
+        <v>6815556677.7906485</v>
       </c>
       <c r="M2" s="1">
-        <v>6101352143.5939369</v>
+        <v>4089334006.6743889</v>
       </c>
       <c r="N2" s="1">
-        <v>4358108673.9956694</v>
+        <v>2920952861.9102778</v>
       </c>
       <c r="O2" s="1">
-        <v>3050676071.7969685</v>
+        <v>2044667003.3371944</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>91</v>
+        <v>380</v>
       </c>
       <c r="B3" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C3" s="1">
         <v>755464100</v>
       </c>
       <c r="D3" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E3" s="1">
-        <v>60584789853.406151</v>
+        <v>40605989558.376778</v>
       </c>
       <c r="F3" s="1">
-        <v>0.51122198685314246</v>
+        <v>0.51122198685314235</v>
       </c>
       <c r="G3" s="1">
-        <v>30972276641.938396</v>
+        <v>20758674660.171329</v>
       </c>
       <c r="H3" s="1">
-        <v>29612513211.467762</v>
+        <v>19847314898.205448</v>
       </c>
       <c r="I3" s="1">
         <v>0.4830000102519989</v>
       </c>
       <c r="J3" s="1">
-        <v>29262454120.310371</v>
+        <v>19612693372.988544</v>
       </c>
       <c r="K3" s="1">
-        <v>20648184427.958931</v>
+        <v>13839116440.11422</v>
       </c>
       <c r="L3" s="1">
-        <v>10324092213.979465</v>
+        <v>6919558220.0571098</v>
       </c>
       <c r="M3" s="1">
-        <v>6194455328.3876791</v>
+        <v>4151734932.034266</v>
       </c>
       <c r="N3" s="1">
-        <v>4424610948.8483419</v>
+        <v>2965524951.4530473</v>
       </c>
       <c r="O3" s="1">
-        <v>3097227664.1938396</v>
+        <v>2075867466.017133</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>92</v>
+        <v>381</v>
       </c>
       <c r="B4" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C4" s="1">
         <v>853582000</v>
       </c>
       <c r="D4" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E4" s="1">
-        <v>68453399827.536652</v>
+        <v>45879799952.397964</v>
       </c>
       <c r="F4" s="1">
-        <v>0.49346782004997725</v>
+        <v>0.4934678200499773</v>
       </c>
       <c r="G4" s="1">
-        <v>33779549987.903999</v>
+        <v>22640204866.838875</v>
       </c>
       <c r="H4" s="1">
-        <v>34673849839.632652</v>
+        <v>23239595085.55909</v>
       </c>
       <c r="I4" s="1">
         <v>0.46599999070167542</v>
       </c>
       <c r="J4" s="1">
-        <v>31899283683.13015</v>
+        <v>21379986351.212181</v>
       </c>
       <c r="K4" s="1">
-        <v>22519699991.936001</v>
+        <v>15093469911.225916</v>
       </c>
       <c r="L4" s="1">
-        <v>11259849995.968</v>
+        <v>7546734955.612958</v>
       </c>
       <c r="M4" s="1">
-        <v>6755909997.5808001</v>
+        <v>4528040973.367775</v>
       </c>
       <c r="N4" s="1">
-        <v>4825649998.2720003</v>
+        <v>3234314980.9769821</v>
       </c>
       <c r="O4" s="1">
-        <v>3377954998.7904</v>
+        <v>2264020486.6838875</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>93</v>
+        <v>382</v>
       </c>
       <c r="B5" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C5" s="1">
         <v>934161000</v>
       </c>
       <c r="D5" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E5" s="1">
-        <v>74915469675.194016</v>
+        <v>50210899249.67025</v>
       </c>
       <c r="F5" s="1">
-        <v>0.48115721201726941</v>
+        <v>0.48115721201726946</v>
       </c>
       <c r="G5" s="1">
-        <v>36046118525.880646</v>
+        <v>24159336295.851345</v>
       </c>
       <c r="H5" s="1">
-        <v>38869351149.31337</v>
+        <v>26051562953.818916</v>
       </c>
       <c r="I5" s="1">
         <v>0.45399999618530273</v>
       </c>
       <c r="J5" s="1">
-        <v>34011622946.758247</v>
+        <v>22795748067.810913</v>
       </c>
       <c r="K5" s="1">
-        <v>24030745683.920429</v>
+        <v>16106224197.23423</v>
       </c>
       <c r="L5" s="1">
-        <v>12015372841.960215</v>
+        <v>8053112098.617115</v>
       </c>
       <c r="M5" s="1">
-        <v>7209223705.1761293</v>
+        <v>4831867259.170269</v>
       </c>
       <c r="N5" s="1">
-        <v>5149445503.6972351</v>
+        <v>3451333756.5501924</v>
       </c>
       <c r="O5" s="1">
-        <v>3604611852.5880647</v>
+        <v>2415933629.5851345</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>383</v>
       </c>
       <c r="B6" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C6" s="1">
         <v>1004399000</v>
       </c>
       <c r="D6" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E6" s="1">
-        <v>80548238286.864044</v>
+        <v>53986172614.21698</v>
       </c>
       <c r="F6" s="1">
-        <v>0.46834795605222707</v>
+        <v>0.46834795605222718</v>
       </c>
       <c r="G6" s="1">
-        <v>37724602765.260513</v>
+        <v>25284313598.951244</v>
       </c>
       <c r="H6" s="1">
-        <v>42823635521.603546</v>
+        <v>28701859015.265739</v>
       </c>
       <c r="I6" s="1">
         <v>0.43700000643730164</v>
       </c>
       <c r="J6" s="1">
-        <v>35199580649.872894</v>
+        <v>23591957779.938099</v>
       </c>
       <c r="K6" s="1">
-        <v>25149735176.840343</v>
+        <v>16856209065.967497</v>
       </c>
       <c r="L6" s="1">
-        <v>12574867588.420172</v>
+        <v>8428104532.9837484</v>
       </c>
       <c r="M6" s="1">
-        <v>7544920553.052103</v>
+        <v>5056862719.7902489</v>
       </c>
       <c r="N6" s="1">
-        <v>5389228966.4657879</v>
+        <v>3612044799.8501778</v>
       </c>
       <c r="O6" s="1">
-        <v>3772460276.5260515</v>
+        <v>2528431359.8951244</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>95</v>
+        <v>384</v>
       </c>
       <c r="B7" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C7" s="1">
         <v>1032567200</v>
       </c>
       <c r="D7" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E7" s="1">
-        <v>82807200000</v>
+        <v>55500205690.147751</v>
       </c>
       <c r="F7" s="1">
-        <v>0.4317008563507454</v>
+        <v>0.43170085635074545</v>
       </c>
       <c r="G7" s="1">
-        <v>35747939152.007446</v>
+        <v>23959486324.0793</v>
       </c>
       <c r="H7" s="1">
-        <v>47059260847.992554</v>
+        <v>31540719366.068459</v>
       </c>
       <c r="I7" s="1">
         <v>0.40099999308586121</v>
       </c>
       <c r="J7" s="1">
-        <v>33205686627.459526</v>
+        <v>22255582098.013123</v>
       </c>
       <c r="K7" s="1">
-        <v>23831959434.671631</v>
+        <v>15972990882.719534</v>
       </c>
       <c r="L7" s="1">
-        <v>11915979717.335815</v>
+        <v>7986495441.359767</v>
       </c>
       <c r="M7" s="1">
-        <v>7149587830.4014893</v>
+        <v>4791897264.8158598</v>
       </c>
       <c r="N7" s="1">
-        <v>5106848450.2867785</v>
+        <v>3422783760.582757</v>
       </c>
       <c r="O7" s="1">
-        <v>3574793915.2007446</v>
+        <v>2395948632.4079299</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>96</v>
+        <v>385</v>
       </c>
       <c r="B8" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C8" s="1">
         <v>1172617000</v>
       </c>
       <c r="D8" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E8" s="1">
-        <v>94038557918.94223</v>
+        <v>63027844285.354004</v>
       </c>
       <c r="F8" s="1">
-        <v>0.4358773788827312</v>
+        <v>0.43587737888273131</v>
       </c>
       <c r="G8" s="1">
-        <v>40989280139.620445</v>
+        <v>27472411563.729038</v>
       </c>
       <c r="H8" s="1">
-        <v>53049277779.32177</v>
+        <v>35555432721.624962</v>
       </c>
       <c r="I8" s="1">
         <v>0.40299999713897705</v>
       </c>
       <c r="J8" s="1">
-        <v>37897538572.287247</v>
+        <v>25400221066.673553</v>
       </c>
       <c r="K8" s="1">
-        <v>27326186759.746964</v>
+        <v>18314941042.486027</v>
       </c>
       <c r="L8" s="1">
-        <v>13663093379.873482</v>
+        <v>9157470521.2430134</v>
       </c>
       <c r="M8" s="1">
-        <v>8197856027.9240894</v>
+        <v>5494482312.7458076</v>
       </c>
       <c r="N8" s="1">
-        <v>5855611448.5172062</v>
+        <v>3924630223.3898625</v>
       </c>
       <c r="O8" s="1">
-        <v>4098928013.9620447</v>
+        <v>2747241156.3729038</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>386</v>
       </c>
       <c r="B9" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C9" s="1">
         <v>1309400000</v>
       </c>
       <c r="D9" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E9" s="1">
-        <v>105007933314.17075</v>
+        <v>70379893270.558533</v>
       </c>
       <c r="F9" s="1">
         <v>0.41915306664806423</v>
       </c>
       <c r="G9" s="1">
-        <v>44014397271.010094</v>
+        <v>29499948094.718067</v>
       </c>
       <c r="H9" s="1">
-        <v>60993536043.160645</v>
+        <v>40879945175.840462</v>
       </c>
       <c r="I9" s="1">
         <v>0.38899999856948853</v>
       </c>
       <c r="J9" s="1">
-        <v>40848085908.997368</v>
+        <v>27377778381.568024</v>
       </c>
       <c r="K9" s="1">
-        <v>29342931514.006729</v>
+        <v>19666632063.145378</v>
       </c>
       <c r="L9" s="1">
-        <v>14671465757.003365</v>
+        <v>9833316031.5726891</v>
       </c>
       <c r="M9" s="1">
-        <v>8802879454.2020187</v>
+        <v>5899989618.9436131</v>
       </c>
       <c r="N9" s="1">
-        <v>6287771038.7157278</v>
+        <v>4214278299.2454381</v>
       </c>
       <c r="O9" s="1">
-        <v>4401439727.1010094</v>
+        <v>2949994809.4718065</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>98</v>
+        <v>387</v>
       </c>
       <c r="B10" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C10" s="1">
         <v>1418700000</v>
       </c>
       <c r="D10" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E10" s="1">
-        <v>113773296924.40356</v>
+        <v>76254738493.158234</v>
       </c>
       <c r="F10" s="1">
-        <v>0.40013900913025569</v>
+        <v>0.40013900913025563</v>
       </c>
       <c r="G10" s="1">
-        <v>45525134296.81321</v>
+        <v>30512495502.139099</v>
       </c>
       <c r="H10" s="1">
-        <v>68248162627.590363</v>
+        <v>45742242991.019135</v>
       </c>
       <c r="I10" s="1">
         <v>0.37599998712539673</v>
       </c>
       <c r="J10" s="1">
-        <v>42778758178.78968</v>
+        <v>28671780691.67799</v>
       </c>
       <c r="K10" s="1">
-        <v>30350089531.208805</v>
+        <v>20341663668.092731</v>
       </c>
       <c r="L10" s="1">
-        <v>15175044765.604403</v>
+        <v>10170831834.046366</v>
       </c>
       <c r="M10" s="1">
-        <v>9105026859.3626423</v>
+        <v>6102499100.4278202</v>
       </c>
       <c r="N10" s="1">
-        <v>6503590613.8304586</v>
+        <v>4358927928.8770142</v>
       </c>
       <c r="O10" s="1">
-        <v>4552513429.6813211</v>
+        <v>3051249550.2139101</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>99</v>
+        <v>388</v>
       </c>
       <c r="B11" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C11" s="1">
         <v>1500800000</v>
       </c>
       <c r="D11" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E11" s="1">
-        <v>120357344064.38632</v>
+        <v>80667591126.053345</v>
       </c>
       <c r="F11" s="1">
-        <v>0.37774737643991424</v>
+        <v>0.37774737643991413</v>
       </c>
       <c r="G11" s="1">
-        <v>45464670955.598015</v>
+        <v>30471970911.594349</v>
       </c>
       <c r="H11" s="1">
-        <v>74892673108.7883</v>
+        <v>50195620214.458984</v>
       </c>
       <c r="I11" s="1">
         <v>0.35199999809265137</v>
       </c>
       <c r="J11" s="1">
-        <v>42365784881.100571</v>
+        <v>28394991922.509556</v>
       </c>
       <c r="K11" s="1">
-        <v>30309780637.065342</v>
+        <v>20314647274.396233</v>
       </c>
       <c r="L11" s="1">
-        <v>15154890318.532671</v>
+        <v>10157323637.198116</v>
       </c>
       <c r="M11" s="1">
-        <v>9092934191.1196022</v>
+        <v>6094394182.3188696</v>
       </c>
       <c r="N11" s="1">
-        <v>6494952993.6568594</v>
+        <v>4353138701.6563358</v>
       </c>
       <c r="O11" s="1">
-        <v>4546467095.5598011</v>
+        <v>3047197091.1594348</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>100</v>
+        <v>389</v>
       </c>
       <c r="B12" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C12" s="1">
         <v>1567700000</v>
       </c>
       <c r="D12" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E12" s="1">
-        <v>125722420235.69992</v>
+        <v>84263447899.99588</v>
       </c>
       <c r="F12" s="1">
-        <v>0.3796082112765885</v>
+        <v>0.37960821127658861</v>
       </c>
       <c r="G12" s="1">
-        <v>47725263063.037621</v>
+        <v>31987096733.315453</v>
       </c>
       <c r="H12" s="1">
-        <v>77997157172.662292</v>
+        <v>52276351166.680435</v>
       </c>
       <c r="I12" s="1">
         <v>0.35499998927116394</v>
       </c>
       <c r="J12" s="1">
-        <v>44631457834.818237</v>
+        <v>29913523100.449818</v>
       </c>
       <c r="K12" s="1">
-        <v>31816842042.025082</v>
+        <v>21324731155.543636</v>
       </c>
       <c r="L12" s="1">
-        <v>15908421021.012541</v>
+        <v>10662365577.771818</v>
       </c>
       <c r="M12" s="1">
-        <v>9545052612.6075249</v>
+        <v>6397419346.6630907</v>
       </c>
       <c r="N12" s="1">
-        <v>6817894723.2910891</v>
+        <v>4569585247.6164932</v>
       </c>
       <c r="O12" s="1">
-        <v>4772526306.3037624</v>
+        <v>3198709673.3315454</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>101</v>
+        <v>390</v>
       </c>
       <c r="B13" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C13" s="1">
         <v>1612500000</v>
       </c>
       <c r="D13" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E13" s="1">
-        <v>129315176774.93533</v>
+        <v>86671435694.803436</v>
       </c>
       <c r="F13" s="1">
-        <v>0.35699156344037641</v>
+        <v>0.35699156344037658</v>
       </c>
       <c r="G13" s="1">
-        <v>46164427133.45282</v>
+        <v>30940971334.30994</v>
       </c>
       <c r="H13" s="1">
-        <v>83150749641.482498</v>
+        <v>55730464360.493515</v>
       </c>
       <c r="I13" s="1">
         <v>0.33300000429153442</v>
       </c>
       <c r="J13" s="1">
-        <v>43061954421.014</v>
+        <v>28861588458.322994</v>
       </c>
       <c r="K13" s="1">
-        <v>30776284755.635212</v>
+        <v>20627314222.873295</v>
       </c>
       <c r="L13" s="1">
-        <v>15388142377.817606</v>
+        <v>10313657111.436647</v>
       </c>
       <c r="M13" s="1">
-        <v>9232885426.6905632</v>
+        <v>6188194266.8619881</v>
       </c>
       <c r="N13" s="1">
-        <v>6594918161.9218311</v>
+        <v>4420138762.0442772</v>
       </c>
       <c r="O13" s="1">
-        <v>4616442713.3452816</v>
+        <v>3094097133.430994</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>102</v>
+        <v>391</v>
       </c>
       <c r="B14" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C14" s="1">
         <v>1713700000</v>
       </c>
       <c r="D14" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E14" s="1">
-        <v>137430957171.60103</v>
+        <v>92110908124.145523</v>
       </c>
       <c r="F14" s="1">
-        <v>0.34094501713251135</v>
+        <v>0.34094501713251141</v>
       </c>
       <c r="G14" s="1">
-        <v>46856400047.408943</v>
+        <v>31404755148.477982</v>
       </c>
       <c r="H14" s="1">
-        <v>90574557124.192078</v>
+        <v>60706152975.667549</v>
       </c>
       <c r="I14" s="1">
         <v>0.31400001049041748</v>
       </c>
       <c r="J14" s="1">
-        <v>43153321993.590836</v>
+        <v>28922826117.263577</v>
       </c>
       <c r="K14" s="1">
-        <v>31237600031.605961</v>
+        <v>20936503432.318653</v>
       </c>
       <c r="L14" s="1">
-        <v>15618800015.80298</v>
+        <v>10468251716.159327</v>
       </c>
       <c r="M14" s="1">
-        <v>9371280009.4817886</v>
+        <v>6280951029.6955967</v>
       </c>
       <c r="N14" s="1">
-        <v>6693771435.3441343</v>
+        <v>4486393592.6397114</v>
       </c>
       <c r="O14" s="1">
-        <v>4685640004.7408943</v>
+        <v>3140475514.8477983</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>103</v>
+        <v>392</v>
       </c>
       <c r="B15" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C15" s="1">
         <v>1792800000</v>
       </c>
       <c r="D15" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E15" s="1">
-        <v>143774417936.18857</v>
+        <v>96362511574.352631</v>
       </c>
       <c r="F15" s="1">
         <v>0.32853097494770572</v>
       </c>
       <c r="G15" s="1">
-        <v>47234349697.114937</v>
+        <v>31658069875.931648</v>
       </c>
       <c r="H15" s="1">
-        <v>96540068239.073624</v>
+        <v>64704441698.420975</v>
       </c>
       <c r="I15" s="1">
         <v>0.3059999942779541</v>
       </c>
       <c r="J15" s="1">
-        <v>43994971065.789886</v>
+        <v>29486927990.361191</v>
       </c>
       <c r="K15" s="1">
-        <v>31489566464.74329</v>
+        <v>21105379917.287766</v>
       </c>
       <c r="L15" s="1">
-        <v>15744783232.371645</v>
+        <v>10552689958.643883</v>
       </c>
       <c r="M15" s="1">
-        <v>9446869939.422987</v>
+        <v>6331613975.1863298</v>
       </c>
       <c r="N15" s="1">
-        <v>6747764242.4449911</v>
+        <v>4522581410.8473787</v>
       </c>
       <c r="O15" s="1">
-        <v>4723434969.7114935</v>
+        <v>3165806987.5931649</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>104</v>
+        <v>393</v>
       </c>
       <c r="B16" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C16" s="1">
         <v>1912900000</v>
       </c>
       <c r="D16" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E16" s="1">
-        <v>153405892497.84421</v>
+        <v>102817853854.62915</v>
       </c>
       <c r="F16" s="1">
         <v>0.35015308008664348</v>
       </c>
       <c r="G16" s="1">
-        <v>53715545761.560661</v>
+        <v>36001988215.096764</v>
       </c>
       <c r="H16" s="1">
-        <v>99690346736.283539</v>
+        <v>66815865639.532379</v>
       </c>
       <c r="I16" s="1">
         <v>0.33000001311302185</v>
       </c>
       <c r="J16" s="1">
-        <v>50623946535.903412</v>
+        <v>33929893120.280384</v>
       </c>
       <c r="K16" s="1">
-        <v>35810363841.040443</v>
+        <v>24001325476.731174</v>
       </c>
       <c r="L16" s="1">
-        <v>17905181920.520222</v>
+        <v>12000662738.365587</v>
       </c>
       <c r="M16" s="1">
-        <v>10743109152.312132</v>
+        <v>7200397643.0193529</v>
       </c>
       <c r="N16" s="1">
-        <v>7673649394.508666</v>
+        <v>5143141173.5852518</v>
       </c>
       <c r="O16" s="1">
-        <v>5371554576.1560659</v>
+        <v>3600198821.5096765</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>105</v>
+        <v>394</v>
       </c>
       <c r="B17" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C17" s="1">
         <v>1968100000</v>
       </c>
       <c r="D17" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E17" s="1">
-        <v>157832681805.11642</v>
+        <v>105784838816.08847</v>
       </c>
       <c r="F17" s="1">
-        <v>0.35752244968095037</v>
+        <v>0.35752244968095032</v>
       </c>
       <c r="G17" s="1">
-        <v>56428727038.679184</v>
+        <v>37820454712.632431</v>
       </c>
       <c r="H17" s="1">
-        <v>101403954766.43724</v>
+        <v>67964384103.456017</v>
       </c>
       <c r="I17" s="1">
         <v>0.33899998664855957</v>
       </c>
       <c r="J17" s="1">
-        <v>53505277024.640816</v>
+        <v>35861058946.274017</v>
       </c>
       <c r="K17" s="1">
-        <v>37619151359.119453</v>
+        <v>25213636475.088287</v>
       </c>
       <c r="L17" s="1">
-        <v>18809575679.559727</v>
+        <v>12606818237.544144</v>
       </c>
       <c r="M17" s="1">
-        <v>11285745407.735836</v>
+        <v>7564090942.5264864</v>
       </c>
       <c r="N17" s="1">
-        <v>8061246719.8113117</v>
+        <v>5402922101.8046331</v>
       </c>
       <c r="O17" s="1">
-        <v>5642872703.867918</v>
+        <v>3782045471.2632432</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>106</v>
+        <v>395</v>
       </c>
       <c r="B18" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C18" s="1">
         <v>1986400000</v>
       </c>
       <c r="D18" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E18" s="1">
-        <v>159300258695.02731</v>
+        <v>106768458830.48531</v>
       </c>
       <c r="F18" s="1">
-        <v>0.35235661559761849</v>
+        <v>0.35235661559761855</v>
       </c>
       <c r="G18" s="1">
-        <v>56130500017.604919</v>
+        <v>37620572806.083473</v>
       </c>
       <c r="H18" s="1">
-        <v>103169758677.42239</v>
+        <v>69147886024.40184</v>
       </c>
       <c r="I18" s="1">
         <v>0.335999995470047</v>
       </c>
       <c r="J18" s="1">
-        <v>53524886199.906494</v>
+        <v>35874201683.386963</v>
       </c>
       <c r="K18" s="1">
-        <v>37420333345.069946</v>
+        <v>25080381870.722317</v>
       </c>
       <c r="L18" s="1">
-        <v>18710166672.534973</v>
+        <v>12540190935.361158</v>
       </c>
       <c r="M18" s="1">
-        <v>11226100003.520985</v>
+        <v>7524114561.2166948</v>
       </c>
       <c r="N18" s="1">
-        <v>8018642859.6578455</v>
+        <v>5374367543.7262106</v>
       </c>
       <c r="O18" s="1">
-        <v>5613050001.7604923</v>
+        <v>3762057280.6083474</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>107</v>
+        <v>396</v>
       </c>
       <c r="B19" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C19" s="1">
         <v>1991300000</v>
       </c>
       <c r="D19" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E19" s="1">
-        <v>159693216441.5062</v>
+        <v>107031832495.54239</v>
       </c>
       <c r="F19" s="1">
         <v>0.32429018551647909</v>
       </c>
       <c r="G19" s="1">
-        <v>51786942785.539291</v>
+        <v>34709372816.148155</v>
       </c>
       <c r="H19" s="1">
-        <v>107906273655.96689</v>
+        <v>72322459679.394226</v>
       </c>
       <c r="I19" s="1">
         <v>0.30500000715255737</v>
       </c>
       <c r="J19" s="1">
-        <v>48706432156.874283</v>
+        <v>32644709676.69175</v>
       </c>
       <c r="K19" s="1">
-        <v>34524628523.692863</v>
+        <v>23139581877.432102</v>
       </c>
       <c r="L19" s="1">
-        <v>17262314261.846432</v>
+        <v>11569790938.716051</v>
       </c>
       <c r="M19" s="1">
-        <v>10357388557.107859</v>
+        <v>6941874563.2296314</v>
       </c>
       <c r="N19" s="1">
-        <v>7398134683.6484699</v>
+        <v>4958481830.8783083</v>
       </c>
       <c r="O19" s="1">
-        <v>5178694278.5539293</v>
+        <v>3470937281.6148157</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>108</v>
+        <v>397</v>
       </c>
       <c r="B20" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C20" s="1">
         <v>2033000000</v>
       </c>
       <c r="D20" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E20" s="1">
-        <v>163037367059.49985</v>
+        <v>109273196134.90567</v>
       </c>
       <c r="F20" s="1">
         <v>0.32675121827917591</v>
       </c>
       <c r="G20" s="1">
-        <v>53272658311.720764</v>
+        <v>35705149962.339767</v>
       </c>
       <c r="H20" s="1">
-        <v>109764708747.7791</v>
+        <v>73568046172.565918</v>
       </c>
       <c r="I20" s="1">
         <v>0.30700001120567322</v>
       </c>
       <c r="J20" s="1">
-        <v>50052473514.209908</v>
+        <v>33546872437.895767</v>
       </c>
       <c r="K20" s="1">
-        <v>35515105541.147179</v>
+        <v>23803433308.226513</v>
       </c>
       <c r="L20" s="1">
-        <v>17757552770.573589</v>
+        <v>11901716654.113256</v>
       </c>
       <c r="M20" s="1">
-        <v>10654531662.344152</v>
+        <v>7141029992.4679537</v>
       </c>
       <c r="N20" s="1">
-        <v>7610379758.8172522</v>
+        <v>5100735708.9056807</v>
       </c>
       <c r="O20" s="1">
-        <v>5327265831.1720762</v>
+        <v>3570514996.2339768</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>109</v>
+        <v>398</v>
       </c>
       <c r="B21" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C21" s="1">
         <v>2051100000</v>
       </c>
       <c r="D21" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E21" s="1">
-        <v>164488904857.71774</v>
+        <v>110246066203.78998</v>
       </c>
       <c r="F21" s="1">
-        <v>0.32450600019122461</v>
+        <v>0.32450600019122472</v>
       </c>
       <c r="G21" s="1">
-        <v>53377636591.212883</v>
+        <v>35775509980.608841</v>
       </c>
       <c r="H21" s="1">
-        <v>111111268266.50484</v>
+        <v>74470556223.181137</v>
       </c>
       <c r="I21" s="1">
         <v>0.30799999833106995</v>
       </c>
       <c r="J21" s="1">
-        <v>50662582421.656586</v>
+        <v>33955788206.774342</v>
       </c>
       <c r="K21" s="1">
-        <v>35585091060.808586</v>
+        <v>23850339987.072559</v>
       </c>
       <c r="L21" s="1">
-        <v>17792545530.404293</v>
+        <v>11925169993.53628</v>
       </c>
       <c r="M21" s="1">
-        <v>10675527318.242577</v>
+        <v>7155101996.121768</v>
       </c>
       <c r="N21" s="1">
-        <v>7625376655.8875551</v>
+        <v>5110787140.086977</v>
       </c>
       <c r="O21" s="1">
-        <v>5337763659.1212883</v>
+        <v>3577550998.060884</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>110</v>
+        <v>399</v>
       </c>
       <c r="B22" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C22" s="1">
         <v>2220500000</v>
       </c>
       <c r="D22" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E22" s="1">
-        <v>178074015521.70163</v>
+        <v>119351270052.90608</v>
       </c>
       <c r="F22" s="1">
-        <v>0.32575769005423599</v>
+        <v>0.32575769005423594</v>
       </c>
       <c r="G22" s="1">
-        <v>58008979955.031685</v>
+        <v>38879594037.473991</v>
       </c>
       <c r="H22" s="1">
-        <v>120065035566.66995</v>
+        <v>80471676015.432083</v>
       </c>
       <c r="I22" s="1">
         <v>0.31000000238418579</v>
       </c>
       <c r="J22" s="1">
-        <v>55202945236.28904</v>
+        <v>36998894000.95649</v>
       </c>
       <c r="K22" s="1">
-        <v>38672653303.354454</v>
+        <v>25919729358.315994</v>
       </c>
       <c r="L22" s="1">
-        <v>19336326651.677227</v>
+        <v>12959864679.157997</v>
       </c>
       <c r="M22" s="1">
-        <v>11601795991.006336</v>
+        <v>7775918807.4947987</v>
       </c>
       <c r="N22" s="1">
-        <v>8286997136.4330978</v>
+        <v>5554227719.639142</v>
       </c>
       <c r="O22" s="1">
-        <v>5800897995.5031681</v>
+        <v>3887959403.7473993</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>111</v>
+        <v>400</v>
       </c>
       <c r="B23" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C23" s="1">
         <v>2327000000</v>
       </c>
       <c r="D23" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E23" s="1">
-        <v>186614831848.23224</v>
+        <v>125075616038.33031</v>
       </c>
       <c r="F23" s="1">
-        <v>0.33278283103433459</v>
+        <v>0.33278283103433448</v>
       </c>
       <c r="G23" s="1">
-        <v>62102212055.451027</v>
+        <v>41623017598.598969</v>
       </c>
       <c r="H23" s="1">
-        <v>124512619792.78122</v>
+        <v>83452598439.731339</v>
       </c>
       <c r="I23" s="1">
         <v>0.31700000166893005</v>
       </c>
       <c r="J23" s="1">
-        <v>59156902007.336723</v>
+        <v>39648970492.893166</v>
       </c>
       <c r="K23" s="1">
-        <v>41401474703.634018</v>
+        <v>27748678399.065979</v>
       </c>
       <c r="L23" s="1">
-        <v>20700737351.817009</v>
+        <v>13874339199.53299</v>
       </c>
       <c r="M23" s="1">
-        <v>12420442411.090206</v>
+        <v>8324603519.7197933</v>
       </c>
       <c r="N23" s="1">
-        <v>8871744579.3501472</v>
+        <v>5946145371.2284241</v>
       </c>
       <c r="O23" s="1">
-        <v>6210221205.5451031</v>
+        <v>4162301759.8598967</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>112</v>
+        <v>401</v>
       </c>
       <c r="B24" t="s">
-        <v>114</v>
+        <v>403</v>
       </c>
       <c r="C24" s="1">
         <v>2389100000</v>
       </c>
       <c r="D24" s="1">
-        <v>80.195458465076172</v>
+        <v>53.749727562668802</v>
       </c>
       <c r="E24" s="1">
-        <v>191594969818.91348</v>
+        <v>128413474119.97203</v>
       </c>
       <c r="F24" s="1">
-        <v>0.31937202175367413</v>
+        <v>0.31937202175367424</v>
       </c>
       <c r="G24" s="1">
-        <v>61190072868.900574</v>
+        <v>41011670850.108589</v>
       </c>
       <c r="H24" s="1">
-        <v>130404896950.01288</v>
+        <v>87401803269.863464</v>
       </c>
       <c r="I24" s="1">
         <v>0.30500000715255737</v>
       </c>
       <c r="J24" s="1">
-        <v>58436467165.162628</v>
+        <v>39166110525.07621</v>
       </c>
       <c r="K24" s="1">
-        <v>40793381912.60038</v>
+        <v>27341113900.072392</v>
       </c>
       <c r="L24" s="1">
-        <v>20396690956.30019</v>
+        <v>13670556950.036196</v>
       </c>
       <c r="M24" s="1">
-        <v>12238014573.780115</v>
+        <v>8202334170.021718</v>
       </c>
       <c r="N24" s="1">
-        <v>8741438981.2715111</v>
+        <v>5858810121.4440842</v>
       </c>
       <c r="O24" s="1">
-        <v>6119007286.8900576</v>
+        <v>4101167085.010859</v>
       </c>
     </row>
   </sheetData>

</xml_diff>